<commit_message>
corpus: 127 finite-element and seepage workbooks no longer carry a surface no page runs
The loader no longer requires a failure surface, so the circles and
non-circular surfaces the builders wrote only to satisfy it are gone from
every workbook that nothing runs a limit-equilibrium analysis on: the
GeoStudio seepage cases, the RS2 groundwater set, the RS2 finite element
rows, the Griffiths and Torggler models, the walls and the block-wall
tutorial's part-3 files. Rebuilt through their builders, which write the
current template; what the loader reads is unchanged except the removed
surface. The corpus circles, rebuild, index, template-sync and preflight
checks pass. Five files with no builder keep theirs for now, as do the
models a limit-equilibrium run or a tutorial reads.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XjjT2aBxw8gY7EFdpoUcpj
</commit_message>
<xml_diff>
--- a/docs/tutorials/files/xslope_base_geotextile_bonded.xlsx
+++ b/docs/tutorials/files/xslope_base_geotextile_bonded.xlsx
@@ -13257,20 +13257,10 @@
       <c r="A3" s="3">
         <v>1</v>
       </c>
-      <c r="B3" s="3">
-        <v>30.0</v>
-      </c>
-      <c r="C3" s="3">
-        <v>15.0</v>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>Depth</t>
-        </is>
-      </c>
-      <c r="E3" s="3">
-        <v>-4.0</v>
-      </c>
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3"/>
       <c r="F3" s="3"/>
       <c r="G3" s="3"/>
       <c r="H3" s="3"/>

</xml_diff>

<commit_message>
builders: write the reinforce Dir/Appl formula results (fill_reinforce_cache) so a rebuilt workbook shows its presets; 21 workbooks rebuilt by their builders (16 move to template v27; loaded models otherwise identical, rebuild check 21/21); LEM-9 sheet renders refreshed
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XjjT2aBxw8gY7EFdpoUcpj
</commit_message>
<xml_diff>
--- a/docs/tutorials/files/xslope_base_geotextile_bonded.xlsx
+++ b/docs/tutorials/files/xslope_base_geotextile_bonded.xlsx
@@ -3776,11 +3776,11 @@
       </c>
       <c r="H3" s="3" t="str">
         <f>IF($G3="","",IFERROR(VLOOKUP($G3,$AH$8:$AJ$11,2,0),""))</f>
-        <v/>
+        <v>Tangent</v>
       </c>
       <c r="I3" s="3" t="str">
         <f t="shared" ref="I3:I32" si="1">IF($G3="","",IFERROR(VLOOKUP($G3,$AH$8:$AJ$11,3,0),""))</f>
-        <v/>
+        <v>Active</v>
       </c>
       <c r="J3" s="3">
         <v>100.0</v>

</xml_diff>